<commit_message>
Mise à jour Excel 2
</commit_message>
<xml_diff>
--- a/uploads/tableau production baptiste-2-a6826d1c.xlsx
+++ b/uploads/tableau production baptiste-2-a6826d1c.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/baptistedavid/Documents/GitHub/book_social_media/uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D6848C5-899B-6944-9361-A5B8B4164169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA5883A-E6B5-024B-B56B-C7BCEABA3741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,15 +31,15 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
+    <customWorkbookView name="Filtre Radio" guid="{8594AFCD-3B41-4B81-B979-5456E2FD0AC3}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Com Sécurité Routière" guid="{26B984F1-F5E8-498D-98EF-4918E7E2C674}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Sanef Solidaire" guid="{E88F7FCD-7F08-4E71-B30C-133DC4379821}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtre Team digitale" guid="{6093BE0E-1F80-46F0-B53B-7F4400F2BFE3}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtre Com Infra" guid="{DB078DD8-52E8-403B-8664-60CFDBD89685}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtre Com Corpo" guid="{8A52195C-3642-4F94-BF33-9498E684A452}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Com corpo" guid="{F190CBEE-8889-45AD-BB7D-398DE1561607}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Com digitale" guid="{9AD516A6-74B3-445D-BF65-F0FC0B0DC784}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
     <customWorkbookView name="Com Radio" guid="{A618CD9D-AFBC-4474-824F-EDA0A02ED83B}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Com digitale" guid="{9AD516A6-74B3-445D-BF65-F0FC0B0DC784}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Com corpo" guid="{F190CBEE-8889-45AD-BB7D-398DE1561607}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtre Com Corpo" guid="{8A52195C-3642-4F94-BF33-9498E684A452}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtre Com Infra" guid="{DB078DD8-52E8-403B-8664-60CFDBD89685}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtre Team digitale" guid="{6093BE0E-1F80-46F0-B53B-7F4400F2BFE3}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Sanef Solidaire" guid="{E88F7FCD-7F08-4E71-B30C-133DC4379821}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Com Sécurité Routière" guid="{26B984F1-F5E8-498D-98EF-4918E7E2C674}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtre Radio" guid="{8594AFCD-3B41-4B81-B979-5456E2FD0AC3}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -4195,17 +4195,17 @@
         <v>121</v>
       </c>
       <c r="J40" s="20">
-        <v>2766</v>
+        <v>30590</v>
       </c>
       <c r="K40" s="21">
-        <v>1758</v>
+        <v>2398</v>
       </c>
       <c r="L40" s="21">
         <v>75</v>
       </c>
       <c r="M40" s="27">
         <f t="shared" si="0"/>
-        <v>4.2662116040955631</v>
+        <v>3.1276063386155126</v>
       </c>
       <c r="N40" s="23"/>
       <c r="O40" s="28"/>
@@ -11163,9 +11163,42 @@
     </filterColumn>
   </autoFilter>
   <customSheetViews>
+    <customSheetView guid="{E88F7FCD-7F08-4E71-B30C-133DC4379821}" filter="1" showAutoFilter="1">
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <autoFilter ref="A1:AB82" xr:uid="{FE94FC31-17EF-144F-A90D-545B6694053D}">
+        <filterColumn colId="3">
+          <filters>
+            <filter val="LinkedIn"/>
+          </filters>
+        </filterColumn>
+      </autoFilter>
+      <extLst>
+        <ext uri="GoogleSheetsCustomDataVersion1">
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="938129022"/>
+        </ext>
+      </extLst>
+    </customSheetView>
+    <customSheetView guid="{A618CD9D-AFBC-4474-824F-EDA0A02ED83B}" filter="1" showAutoFilter="1">
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <autoFilter ref="A1:N282" xr:uid="{7ABF95D0-0CFA-ED4C-88DD-200027017AB2}"/>
+      <extLst>
+        <ext uri="GoogleSheetsCustomDataVersion1">
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="40062235"/>
+        </ext>
+      </extLst>
+    </customSheetView>
+    <customSheetView guid="{F190CBEE-8889-45AD-BB7D-398DE1561607}" filter="1" showAutoFilter="1">
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <autoFilter ref="A1:N282" xr:uid="{BAA9AF62-6A58-5C47-9646-61C27F58C6AF}"/>
+      <extLst>
+        <ext uri="GoogleSheetsCustomDataVersion1">
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1404300964"/>
+        </ext>
+      </extLst>
+    </customSheetView>
     <customSheetView guid="{9AD516A6-74B3-445D-BF65-F0FC0B0DC784}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N282" xr:uid="{83C4A3E8-90B7-4E4D-BA5D-E7D1849F2B7A}">
+      <autoFilter ref="A1:N282" xr:uid="{70480399-F3D7-964F-9728-11863CD39E49}">
         <filterColumn colId="2">
           <filters>
             <filter val="Com digitale"/>
@@ -11175,39 +11208,6 @@
       <extLst>
         <ext uri="GoogleSheetsCustomDataVersion1">
           <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1038187113"/>
-        </ext>
-      </extLst>
-    </customSheetView>
-    <customSheetView guid="{F190CBEE-8889-45AD-BB7D-398DE1561607}" filter="1" showAutoFilter="1">
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N282" xr:uid="{31308174-3CAF-354C-A303-ED9E5E95FAA9}"/>
-      <extLst>
-        <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1404300964"/>
-        </ext>
-      </extLst>
-    </customSheetView>
-    <customSheetView guid="{A618CD9D-AFBC-4474-824F-EDA0A02ED83B}" filter="1" showAutoFilter="1">
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N282" xr:uid="{C95C0AAD-34CB-0B46-A1C4-4E0B74176E9B}"/>
-      <extLst>
-        <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="40062235"/>
-        </ext>
-      </extLst>
-    </customSheetView>
-    <customSheetView guid="{E88F7FCD-7F08-4E71-B30C-133DC4379821}" filter="1" showAutoFilter="1">
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:AB82" xr:uid="{DEBBF716-1E98-BB4E-AD9E-50AAFD675E3E}">
-        <filterColumn colId="3">
-          <filters>
-            <filter val="LinkedIn"/>
-          </filters>
-        </filterColumn>
-      </autoFilter>
-      <extLst>
-        <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="938129022"/>
         </ext>
       </extLst>
     </customSheetView>
@@ -16421,27 +16421,27 @@
   </sheetData>
   <autoFilter ref="A1:N30" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <customSheetViews>
-    <customSheetView guid="{26B984F1-F5E8-498D-98EF-4918E7E2C674}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{8A52195C-3642-4F94-BF33-9498E684A452}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N66" xr:uid="{8DD4847B-DC8F-784B-8572-6B8A14BBEAD5}"/>
+      <autoFilter ref="A1:N66" xr:uid="{DE2D4D54-C2C4-5246-8920-2E73FCE15824}"/>
       <extLst>
         <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1311743053"/>
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="270424754"/>
         </ext>
       </extLst>
     </customSheetView>
-    <customSheetView guid="{6093BE0E-1F80-46F0-B53B-7F4400F2BFE3}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{DB078DD8-52E8-403B-8664-60CFDBD89685}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N230" xr:uid="{EDBF168E-0F12-C944-8277-8998808051AE}"/>
+      <autoFilter ref="A1:N66" xr:uid="{8FC9A773-FB86-0D4B-98DA-8DFA37BD61DD}"/>
       <extLst>
         <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1754472313"/>
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="213558549"/>
         </ext>
       </extLst>
     </customSheetView>
     <customSheetView guid="{8594AFCD-3B41-4B81-B979-5456E2FD0AC3}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N66" xr:uid="{A675F61C-74C3-D942-AE63-98B17F68C681}">
+      <autoFilter ref="A1:N66" xr:uid="{D0345712-8D06-0440-BB66-1E494E87DF55}">
         <filterColumn colId="0">
           <filters blank="1">
             <filter val="December"/>
@@ -16474,21 +16474,21 @@
         </ext>
       </extLst>
     </customSheetView>
-    <customSheetView guid="{DB078DD8-52E8-403B-8664-60CFDBD89685}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{6093BE0E-1F80-46F0-B53B-7F4400F2BFE3}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N66" xr:uid="{D102A5BE-3581-034B-B36C-C1B9D6C0E4A8}"/>
+      <autoFilter ref="A1:N230" xr:uid="{4F69F0A7-7C97-794D-AE08-2BF9D3E3CAE2}"/>
       <extLst>
         <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="213558549"/>
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1754472313"/>
         </ext>
       </extLst>
     </customSheetView>
-    <customSheetView guid="{8A52195C-3642-4F94-BF33-9498E684A452}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{26B984F1-F5E8-498D-98EF-4918E7E2C674}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N66" xr:uid="{CBEEA22F-9369-D84A-BFCB-8B91CA8CCB27}"/>
+      <autoFilter ref="A1:N66" xr:uid="{B95A06F4-02A4-3545-A72E-9E2883E4E26E}"/>
       <extLst>
         <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="270424754"/>
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1311743053"/>
         </ext>
       </extLst>
     </customSheetView>

</xml_diff>

<commit_message>
mise à jour post audience
</commit_message>
<xml_diff>
--- a/uploads/tableau production baptiste-2-a6826d1c.xlsx
+++ b/uploads/tableau production baptiste-2-a6826d1c.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/baptistedavid/Documents/GitHub/book_social_media/uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA5883A-E6B5-024B-B56B-C7BCEABA3741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2695A196-E014-374A-B8DE-E34E0F17F0D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1922,7 +1922,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:AB612"/>
@@ -2057,7 +2057,7 @@
       <c r="AA2" s="25"/>
       <c r="AB2" s="25"/>
     </row>
-    <row r="3" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="3" spans="1:28" ht="55.5" customHeight="1">
       <c r="A3" s="14">
         <v>46023</v>
       </c>
@@ -2171,7 +2171,7 @@
       <c r="AA4" s="25"/>
       <c r="AB4" s="25"/>
     </row>
-    <row r="5" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="5" spans="1:28" ht="55.5" customHeight="1">
       <c r="A5" s="14">
         <v>46023</v>
       </c>
@@ -2228,7 +2228,7 @@
       <c r="AA5" s="25"/>
       <c r="AB5" s="25"/>
     </row>
-    <row r="6" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="6" spans="1:28" ht="55.5" customHeight="1">
       <c r="A6" s="14">
         <v>46023</v>
       </c>
@@ -2285,7 +2285,7 @@
       <c r="AA6" s="25"/>
       <c r="AB6" s="25"/>
     </row>
-    <row r="7" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="7" spans="1:28" ht="55.5" customHeight="1">
       <c r="A7" s="14">
         <v>46023</v>
       </c>
@@ -2342,7 +2342,7 @@
       <c r="AA7" s="25"/>
       <c r="AB7" s="25"/>
     </row>
-    <row r="8" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="8" spans="1:28" ht="55.5" customHeight="1">
       <c r="A8" s="14">
         <v>46023</v>
       </c>
@@ -2399,7 +2399,7 @@
       <c r="AA8" s="25"/>
       <c r="AB8" s="25"/>
     </row>
-    <row r="9" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="9" spans="1:28" ht="55.5" customHeight="1">
       <c r="A9" s="14">
         <v>46023</v>
       </c>
@@ -2456,7 +2456,7 @@
       <c r="AA9" s="25"/>
       <c r="AB9" s="25"/>
     </row>
-    <row r="10" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="10" spans="1:28" ht="55.5" customHeight="1">
       <c r="A10" s="14">
         <v>46054</v>
       </c>
@@ -2513,7 +2513,7 @@
       <c r="AA10" s="25"/>
       <c r="AB10" s="25"/>
     </row>
-    <row r="11" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="11" spans="1:28" ht="55.5" customHeight="1">
       <c r="A11" s="14">
         <v>46054</v>
       </c>
@@ -2741,7 +2741,7 @@
       <c r="AA14" s="25"/>
       <c r="AB14" s="25"/>
     </row>
-    <row r="15" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="15" spans="1:28" ht="55.5" customHeight="1">
       <c r="A15" s="14">
         <v>46054</v>
       </c>
@@ -2798,7 +2798,7 @@
       <c r="AA15" s="28"/>
       <c r="AB15" s="28"/>
     </row>
-    <row r="16" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="16" spans="1:28" ht="55.5" customHeight="1">
       <c r="A16" s="14">
         <v>46054</v>
       </c>
@@ -2855,7 +2855,7 @@
       <c r="AA16" s="28"/>
       <c r="AB16" s="28"/>
     </row>
-    <row r="17" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="17" spans="1:28" ht="55.5" customHeight="1">
       <c r="A17" s="14">
         <v>46054</v>
       </c>
@@ -2969,7 +2969,7 @@
       <c r="AA18" s="25"/>
       <c r="AB18" s="25"/>
     </row>
-    <row r="19" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="19" spans="1:28" ht="55.5" customHeight="1">
       <c r="A19" s="14">
         <v>46054</v>
       </c>
@@ -3026,7 +3026,7 @@
       <c r="AA19" s="25"/>
       <c r="AB19" s="25"/>
     </row>
-    <row r="20" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="20" spans="1:28" ht="55.5" customHeight="1">
       <c r="A20" s="14">
         <v>46054</v>
       </c>
@@ -3197,7 +3197,7 @@
       <c r="AA22" s="28"/>
       <c r="AB22" s="28"/>
     </row>
-    <row r="23" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="23" spans="1:28" ht="55.5" customHeight="1">
       <c r="A23" s="14">
         <v>46054</v>
       </c>
@@ -3254,7 +3254,7 @@
       <c r="AA23" s="28"/>
       <c r="AB23" s="28"/>
     </row>
-    <row r="24" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="24" spans="1:28" ht="55.5" customHeight="1">
       <c r="A24" s="14">
         <v>46054</v>
       </c>
@@ -3311,7 +3311,7 @@
       <c r="AA24" s="28"/>
       <c r="AB24" s="28"/>
     </row>
-    <row r="25" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="25" spans="1:28" ht="55.5" customHeight="1">
       <c r="A25" s="14">
         <v>46054</v>
       </c>
@@ -3368,7 +3368,7 @@
       <c r="AA25" s="28"/>
       <c r="AB25" s="28"/>
     </row>
-    <row r="26" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="26" spans="1:28" ht="55.5" customHeight="1">
       <c r="A26" s="14">
         <v>46054</v>
       </c>
@@ -3425,7 +3425,7 @@
       <c r="AA26" s="28"/>
       <c r="AB26" s="28"/>
     </row>
-    <row r="27" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="27" spans="1:28" ht="55.5" customHeight="1">
       <c r="A27" s="14">
         <v>46082</v>
       </c>
@@ -3482,7 +3482,7 @@
       <c r="AA27" s="28"/>
       <c r="AB27" s="28"/>
     </row>
-    <row r="28" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="28" spans="1:28" ht="55.5" customHeight="1">
       <c r="A28" s="14">
         <v>46082</v>
       </c>
@@ -3539,7 +3539,7 @@
       <c r="AA28" s="28"/>
       <c r="AB28" s="28"/>
     </row>
-    <row r="29" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="29" spans="1:28" ht="55.5" customHeight="1">
       <c r="A29" s="14">
         <v>46082</v>
       </c>
@@ -3596,7 +3596,7 @@
       <c r="AA29" s="28"/>
       <c r="AB29" s="28"/>
     </row>
-    <row r="30" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="30" spans="1:28" ht="55.5" customHeight="1">
       <c r="A30" s="14">
         <v>46082</v>
       </c>
@@ -3653,7 +3653,7 @@
       <c r="AA30" s="28"/>
       <c r="AB30" s="28"/>
     </row>
-    <row r="31" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="31" spans="1:28" ht="55.5" customHeight="1">
       <c r="A31" s="14">
         <v>46082</v>
       </c>
@@ -3710,7 +3710,7 @@
       <c r="AA31" s="25"/>
       <c r="AB31" s="25"/>
     </row>
-    <row r="32" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="32" spans="1:28" ht="55.5" customHeight="1">
       <c r="A32" s="14">
         <v>46082</v>
       </c>
@@ -3767,7 +3767,7 @@
       <c r="AA32" s="28"/>
       <c r="AB32" s="28"/>
     </row>
-    <row r="33" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="33" spans="1:28" ht="55.5" customHeight="1">
       <c r="A33" s="14">
         <v>46082</v>
       </c>
@@ -3824,7 +3824,7 @@
       <c r="AA33" s="28"/>
       <c r="AB33" s="28"/>
     </row>
-    <row r="34" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="34" spans="1:28" ht="55.5" customHeight="1">
       <c r="A34" s="14">
         <v>46082</v>
       </c>
@@ -3995,7 +3995,7 @@
       <c r="AA36" s="28"/>
       <c r="AB36" s="28"/>
     </row>
-    <row r="37" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="37" spans="1:28" ht="55.5" customHeight="1">
       <c r="A37" s="14">
         <v>46082</v>
       </c>
@@ -4109,7 +4109,7 @@
       <c r="AA38" s="28"/>
       <c r="AB38" s="28"/>
     </row>
-    <row r="39" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="39" spans="1:28" ht="55.5" customHeight="1">
       <c r="A39" s="14">
         <v>46082</v>
       </c>
@@ -4223,7 +4223,7 @@
       <c r="AA40" s="28"/>
       <c r="AB40" s="28"/>
     </row>
-    <row r="41" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="41" spans="1:28" ht="55.5" customHeight="1">
       <c r="A41" s="14">
         <v>46082</v>
       </c>
@@ -4394,7 +4394,7 @@
       <c r="AA43" s="28"/>
       <c r="AB43" s="28"/>
     </row>
-    <row r="44" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="44" spans="1:28" ht="55.5" customHeight="1">
       <c r="A44" s="14">
         <v>46082</v>
       </c>
@@ -4508,7 +4508,7 @@
       <c r="AA45" s="28"/>
       <c r="AB45" s="28"/>
     </row>
-    <row r="46" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="46" spans="1:28" ht="55.5" customHeight="1">
       <c r="A46" s="14">
         <v>46082</v>
       </c>
@@ -4565,7 +4565,7 @@
       <c r="AA46" s="28"/>
       <c r="AB46" s="28"/>
     </row>
-    <row r="47" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="47" spans="1:28" ht="55.5" customHeight="1">
       <c r="A47" s="14">
         <v>46082</v>
       </c>
@@ -4622,7 +4622,7 @@
       <c r="AA47" s="28"/>
       <c r="AB47" s="28"/>
     </row>
-    <row r="48" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="48" spans="1:28" ht="55.5" customHeight="1">
       <c r="A48" s="14">
         <v>46082</v>
       </c>
@@ -4679,7 +4679,7 @@
       <c r="AA48" s="28"/>
       <c r="AB48" s="28"/>
     </row>
-    <row r="49" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="49" spans="1:28" ht="55.5" customHeight="1">
       <c r="A49" s="14">
         <v>46082</v>
       </c>
@@ -4731,7 +4731,7 @@
       <c r="AA49" s="28"/>
       <c r="AB49" s="28"/>
     </row>
-    <row r="50" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="50" spans="1:28" ht="55.5" customHeight="1">
       <c r="A50" s="14">
         <v>46082</v>
       </c>
@@ -4788,7 +4788,7 @@
       <c r="AA50" s="28"/>
       <c r="AB50" s="28"/>
     </row>
-    <row r="51" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="51" spans="1:28" ht="55.5" customHeight="1">
       <c r="A51" s="14">
         <v>46113</v>
       </c>
@@ -4845,7 +4845,7 @@
       <c r="AA51" s="25"/>
       <c r="AB51" s="25"/>
     </row>
-    <row r="52" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="52" spans="1:28" ht="55.5" customHeight="1">
       <c r="A52" s="14">
         <v>46113</v>
       </c>
@@ -4961,7 +4961,7 @@
       <c r="AA53" s="25"/>
       <c r="AB53" s="25"/>
     </row>
-    <row r="54" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="54" spans="1:28" ht="55.5" customHeight="1">
       <c r="A54" s="14">
         <v>46113</v>
       </c>
@@ -5018,7 +5018,7 @@
       <c r="AA54" s="25"/>
       <c r="AB54" s="25"/>
     </row>
-    <row r="55" spans="1:28" ht="70.5" hidden="1" customHeight="1">
+    <row r="55" spans="1:28" ht="70.5" customHeight="1">
       <c r="A55" s="14">
         <v>46113</v>
       </c>
@@ -5075,7 +5075,7 @@
       <c r="AA55" s="25"/>
       <c r="AB55" s="25"/>
     </row>
-    <row r="56" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="56" spans="1:28" ht="55.5" customHeight="1">
       <c r="A56" s="14">
         <v>46113</v>
       </c>
@@ -5132,7 +5132,7 @@
       <c r="AA56" s="25"/>
       <c r="AB56" s="25"/>
     </row>
-    <row r="57" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="57" spans="1:28" ht="55.5" customHeight="1">
       <c r="A57" s="14">
         <v>46113</v>
       </c>
@@ -5189,7 +5189,7 @@
       <c r="AA57" s="25"/>
       <c r="AB57" s="25"/>
     </row>
-    <row r="58" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="58" spans="1:28" ht="55.5" customHeight="1">
       <c r="A58" s="14">
         <v>46113</v>
       </c>
@@ -5246,7 +5246,7 @@
       <c r="AA58" s="25"/>
       <c r="AB58" s="25"/>
     </row>
-    <row r="59" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="59" spans="1:28" ht="55.5" customHeight="1">
       <c r="A59" s="14">
         <v>46143</v>
       </c>
@@ -5303,7 +5303,7 @@
       <c r="AA59" s="25"/>
       <c r="AB59" s="25"/>
     </row>
-    <row r="60" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="60" spans="1:28" ht="55.5" customHeight="1">
       <c r="A60" s="14">
         <v>46143</v>
       </c>
@@ -5360,7 +5360,7 @@
       <c r="AA60" s="25"/>
       <c r="AB60" s="25"/>
     </row>
-    <row r="61" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="61" spans="1:28" ht="55.5" customHeight="1">
       <c r="A61" s="14">
         <v>46143</v>
       </c>
@@ -5474,7 +5474,7 @@
       <c r="AA62" s="25"/>
       <c r="AB62" s="25"/>
     </row>
-    <row r="63" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="63" spans="1:28" ht="55.5" customHeight="1">
       <c r="A63" s="14">
         <v>46143</v>
       </c>
@@ -5588,7 +5588,7 @@
       <c r="AA64" s="25"/>
       <c r="AB64" s="25"/>
     </row>
-    <row r="65" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="65" spans="1:28" ht="55.5" customHeight="1">
       <c r="A65" s="14">
         <v>46143</v>
       </c>
@@ -5759,7 +5759,7 @@
       <c r="AA67" s="25"/>
       <c r="AB67" s="25"/>
     </row>
-    <row r="68" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="68" spans="1:28" ht="55.5" customHeight="1">
       <c r="A68" s="14">
         <v>46143</v>
       </c>
@@ -5873,7 +5873,7 @@
       <c r="AA69" s="25"/>
       <c r="AB69" s="25"/>
     </row>
-    <row r="70" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="70" spans="1:28" ht="55.5" customHeight="1">
       <c r="A70" s="14">
         <v>46143</v>
       </c>
@@ -5987,7 +5987,7 @@
       <c r="AA71" s="25"/>
       <c r="AB71" s="25"/>
     </row>
-    <row r="72" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="72" spans="1:28" ht="55.5" customHeight="1">
       <c r="A72" s="14">
         <v>46143</v>
       </c>
@@ -6044,7 +6044,7 @@
       <c r="AA72" s="25"/>
       <c r="AB72" s="25"/>
     </row>
-    <row r="73" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="73" spans="1:28" ht="55.5" customHeight="1">
       <c r="A73" s="14">
         <v>46143</v>
       </c>
@@ -6101,7 +6101,7 @@
       <c r="AA73" s="25"/>
       <c r="AB73" s="25"/>
     </row>
-    <row r="74" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="74" spans="1:28" ht="55.5" customHeight="1">
       <c r="A74" s="14">
         <v>46143</v>
       </c>
@@ -6158,7 +6158,7 @@
       <c r="AA74" s="25"/>
       <c r="AB74" s="25"/>
     </row>
-    <row r="75" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="75" spans="1:28" ht="55.5" customHeight="1">
       <c r="A75" s="14">
         <v>46143</v>
       </c>
@@ -6272,7 +6272,7 @@
       <c r="AA76" s="25"/>
       <c r="AB76" s="25"/>
     </row>
-    <row r="77" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="77" spans="1:28" ht="55.5" customHeight="1">
       <c r="A77" s="14">
         <v>46143</v>
       </c>
@@ -6329,7 +6329,7 @@
       <c r="AA77" s="25"/>
       <c r="AB77" s="25"/>
     </row>
-    <row r="78" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="78" spans="1:28" ht="55.5" customHeight="1">
       <c r="A78" s="14">
         <v>46143</v>
       </c>
@@ -6377,7 +6377,7 @@
       <c r="AA78" s="25"/>
       <c r="AB78" s="25"/>
     </row>
-    <row r="79" spans="1:28" ht="15.75" hidden="1" customHeight="1">
+    <row r="79" spans="1:28" ht="15.75" customHeight="1">
       <c r="A79" s="14">
         <v>46174</v>
       </c>
@@ -6425,7 +6425,7 @@
       <c r="AA79" s="25"/>
       <c r="AB79" s="25"/>
     </row>
-    <row r="80" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="80" spans="1:28" ht="55.5" customHeight="1">
       <c r="A80" s="14">
         <v>46174</v>
       </c>
@@ -6475,7 +6475,7 @@
       <c r="AA80" s="25"/>
       <c r="AB80" s="25"/>
     </row>
-    <row r="81" spans="1:28" s="93" customFormat="1" ht="55.5" hidden="1" customHeight="1">
+    <row r="81" spans="1:28" s="93" customFormat="1" ht="55.5" customHeight="1">
       <c r="A81" s="90" t="s">
         <v>12</v>
       </c>
@@ -6531,7 +6531,7 @@
       <c r="AA81" s="88"/>
       <c r="AB81" s="88"/>
     </row>
-    <row r="82" spans="1:28" ht="55.5" hidden="1" customHeight="1">
+    <row r="82" spans="1:28" ht="55.5" customHeight="1">
       <c r="A82" s="14">
         <v>46174</v>
       </c>
@@ -11148,20 +11148,7 @@
       <c r="N612" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O82" xr:uid="{00000000-0009-0000-0000-000002000000}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="Instagram"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="4">
-      <filters>
-        <filter val="Post"/>
-        <filter val="Quiz"/>
-        <filter val="Reel"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:O82" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <customSheetViews>
     <customSheetView guid="{E88F7FCD-7F08-4E71-B30C-133DC4379821}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>